<commit_message>
Fix preview and 99 limit
</commit_message>
<xml_diff>
--- a/examples/test_contacts.xlsx
+++ b/examples/test_contacts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/smurdoch/w/mail-merge/examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAAD43C6-9CFE-FF42-A193-79B57E2B9272}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7894FCCA-FA76-E743-BEDC-CCF6A122F73F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="16">
   <si>
     <t>email</t>
   </si>
@@ -69,6 +69,18 @@
   </si>
   <si>
     <t>Steven 3 Murdoch</t>
+  </si>
+  <si>
+    <t>FCS</t>
+  </si>
+  <si>
+    <t>AI</t>
+  </si>
+  <si>
+    <t>AC</t>
+  </si>
+  <si>
+    <t>section</t>
   </si>
 </sst>
 </file>
@@ -346,10 +358,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1ED8F166-36A1-E843-93A3-ECA5945FAD3B}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <sheetData>
-    <row r="1" spans="1:3" ht="16" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
@@ -359,8 +371,11 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="D1" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -370,8 +385,11 @@
       <c r="C2" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="D2" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -381,8 +399,11 @@
       <c r="C3" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="D3" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.15">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
@@ -391,6 +412,51 @@
       </c>
       <c r="C4" s="1" t="s">
         <v>11</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A6" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A7" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -398,6 +464,9 @@
     <hyperlink ref="B2" r:id="rId1" xr:uid="{C4D30075-6201-A04E-9E33-CE604A08EF50}"/>
     <hyperlink ref="B3" r:id="rId2" xr:uid="{31DD94E9-4BBE-C54B-9EAA-9F488CD1753F}"/>
     <hyperlink ref="B4" r:id="rId3" xr:uid="{377EC2A5-EB57-3843-BCCA-664BFE349708}"/>
+    <hyperlink ref="B5" r:id="rId4" xr:uid="{A4BA2E58-662D-EF44-890C-733969D12181}"/>
+    <hyperlink ref="B6" r:id="rId5" xr:uid="{045D5230-78FD-9A46-8077-D0E13211C409}"/>
+    <hyperlink ref="B7" r:id="rId6" xr:uid="{42B075E7-F93A-854A-AA4D-D303F6403150}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Set up standalone executable
</commit_message>
<xml_diff>
--- a/examples/test_contacts.xlsx
+++ b/examples/test_contacts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/smurdoch/w/mail-merge/examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7894FCCA-FA76-E743-BEDC-CCF6A122F73F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7EAD1A3-622B-AC47-A2D0-D9B9251EE544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="19">
   <si>
     <t>email</t>
   </si>
@@ -81,6 +81,15 @@
   </si>
   <si>
     <t>section</t>
+  </si>
+  <si>
+    <t>INV1</t>
+  </si>
+  <si>
+    <t>franziska.​murdoch@​rub.​de</t>
+  </si>
+  <si>
+    <t>Steven 4</t>
   </si>
 </sst>
 </file>
@@ -358,7 +367,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1ED8F166-36A1-E843-93A3-ECA5945FAD3B}">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <sheetData>
     <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.25">
@@ -457,6 +466,20 @@
       </c>
       <c r="D7" s="1" t="s">
         <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A8" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Exit cleanly if signing stage succeeds
</commit_message>
<xml_diff>
--- a/examples/test_contacts.xlsx
+++ b/examples/test_contacts.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/smurdoch/w/mail-merge/examples/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/smurdoch/w/MergeMail365/examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7EAD1A3-622B-AC47-A2D0-D9B9251EE544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88E2438B-BB8D-C943-AEEA-ABD4AB8630FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="4" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="5" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="26">
   <si>
     <t>email</t>
   </si>
@@ -90,13 +91,34 @@
   </si>
   <si>
     <t>Steven 4</t>
+  </si>
+  <si>
+    <t>ABC1</t>
+  </si>
+  <si>
+    <t>ABC2</t>
+  </si>
+  <si>
+    <t>ABC3</t>
+  </si>
+  <si>
+    <t>ABC4</t>
+  </si>
+  <si>
+    <t>ABC5</t>
+  </si>
+  <si>
+    <t>ABC6</t>
+  </si>
+  <si>
+    <t>INV1b</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -123,6 +145,12 @@
       <color rgb="FF000000"/>
       <name val="Arial Unicode MS"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -493,4 +521,135 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1274D1D3-AEB9-914B-95A5-3B67AC0F9A2F}">
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <sheetData>
+    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A6" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.15">
+      <c r="A8" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{C49CC857-6714-C54A-A93D-9B7F56A9E160}"/>
+    <hyperlink ref="B3" r:id="rId2" xr:uid="{C49C70F1-3DAC-3D40-8A3F-2FBD8082188C}"/>
+    <hyperlink ref="B4" r:id="rId3" xr:uid="{17C32820-4ED8-4C42-82DF-89802A772D8F}"/>
+    <hyperlink ref="B5" r:id="rId4" xr:uid="{0BF60B2B-78C0-164C-BD2C-41394467D2EE}"/>
+    <hyperlink ref="B6" r:id="rId5" xr:uid="{36AA0B96-34A1-114B-B995-1A75910EEF4F}"/>
+    <hyperlink ref="B7" r:id="rId6" xr:uid="{D8811105-4DE3-E849-AB23-F59AA1D22E06}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>